<commit_message>
Teste do script do github actions
</commit_message>
<xml_diff>
--- a/dados/d_Enderecos.xlsx
+++ b/dados/d_Enderecos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Meu Drive\UFG\2026.1\ESTAGIO OBRIGATORIO\2026.1\ATIVIDADES SEINFRA\BI FATURAS\BI VICTOR\AUXILIARES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Meu Drive\TRABALHO\BOLSA FUNAPE\ATIVIDADES SEINFRA\BI para HTML\BASE GITHUB\faturas-seinfra-ufg\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A90ABED-0B99-4C60-A0A9-1EC6CFAA92BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A60F50CD-6787-4B0C-9DDD-B882899038BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C2B8D48B-2285-4DAE-865B-37B0AD0C50CA}"/>
   </bookViews>
@@ -1158,13 +1158,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1548,7 +1547,7 @@
       <c r="B2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="1" t="s">
         <v>318</v>
       </c>
       <c r="D2" t="s">
@@ -1577,7 +1576,7 @@
       <c r="B3" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="1" t="s">
         <v>344</v>
       </c>
       <c r="D3" t="s">
@@ -1606,7 +1605,7 @@
       <c r="B4" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="1" t="s">
         <v>341</v>
       </c>
       <c r="D4" t="s">
@@ -1635,7 +1634,7 @@
       <c r="B5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="1" t="s">
         <v>312</v>
       </c>
       <c r="D5" t="s">
@@ -1664,7 +1663,7 @@
       <c r="B6" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="1" t="s">
         <v>324</v>
       </c>
       <c r="D6" t="s">
@@ -1693,7 +1692,7 @@
       <c r="B7" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="1" t="s">
         <v>346</v>
       </c>
       <c r="D7" t="s">
@@ -1722,7 +1721,7 @@
       <c r="B8" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="1" t="s">
         <v>328</v>
       </c>
       <c r="D8" t="s">
@@ -1751,7 +1750,7 @@
       <c r="B9" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="1" t="s">
         <v>342</v>
       </c>
       <c r="D9" t="s">
@@ -1780,7 +1779,7 @@
       <c r="B10" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="1" t="s">
         <v>343</v>
       </c>
       <c r="D10" t="s">
@@ -1809,7 +1808,7 @@
       <c r="B11" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="1" t="s">
         <v>327</v>
       </c>
       <c r="D11" t="s">
@@ -1838,7 +1837,7 @@
       <c r="B12" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="1" t="s">
         <v>337</v>
       </c>
       <c r="D12" t="s">
@@ -1867,7 +1866,7 @@
       <c r="B13" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="1" t="s">
         <v>319</v>
       </c>
       <c r="D13" t="s">
@@ -1896,7 +1895,7 @@
       <c r="B14" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="1" t="s">
         <v>338</v>
       </c>
       <c r="D14" t="s">
@@ -1925,7 +1924,7 @@
       <c r="B15" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="1" t="s">
         <v>315</v>
       </c>
       <c r="D15" t="s">
@@ -1954,7 +1953,7 @@
       <c r="B16" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="1" t="s">
         <v>336</v>
       </c>
       <c r="D16" t="s">
@@ -1983,7 +1982,7 @@
       <c r="B17" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="1" t="s">
         <v>352</v>
       </c>
       <c r="D17" t="s">
@@ -2012,7 +2011,7 @@
       <c r="B18" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="1" t="s">
         <v>320</v>
       </c>
       <c r="D18" t="s">
@@ -2041,7 +2040,7 @@
       <c r="B19" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="1" t="s">
         <v>356</v>
       </c>
       <c r="D19" t="s">
@@ -2070,7 +2069,7 @@
       <c r="B20" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="1" t="s">
         <v>333</v>
       </c>
       <c r="D20" t="s">
@@ -2099,7 +2098,7 @@
       <c r="B21" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="1" t="s">
         <v>313</v>
       </c>
       <c r="D21" t="s">
@@ -2128,7 +2127,7 @@
       <c r="B22" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="1" t="s">
         <v>321</v>
       </c>
       <c r="D22" t="s">
@@ -2157,7 +2156,7 @@
       <c r="B23" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="1" t="s">
         <v>326</v>
       </c>
       <c r="D23" t="s">
@@ -2186,7 +2185,7 @@
       <c r="B24" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="1" t="s">
         <v>347</v>
       </c>
       <c r="D24" t="s">
@@ -2215,7 +2214,7 @@
       <c r="B25" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="1" t="s">
         <v>351</v>
       </c>
       <c r="D25" t="s">
@@ -2244,7 +2243,7 @@
       <c r="B26" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="1" t="s">
         <v>349</v>
       </c>
       <c r="D26" t="s">
@@ -2273,7 +2272,7 @@
       <c r="B27" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="1" t="s">
         <v>348</v>
       </c>
       <c r="D27" t="s">
@@ -2302,7 +2301,7 @@
       <c r="B28" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="1" t="s">
         <v>350</v>
       </c>
       <c r="D28" t="s">
@@ -2331,7 +2330,7 @@
       <c r="B29" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="1" t="s">
         <v>331</v>
       </c>
       <c r="D29" t="s">
@@ -2360,7 +2359,7 @@
       <c r="B30" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="1" t="s">
         <v>334</v>
       </c>
       <c r="D30" t="s">
@@ -2389,7 +2388,7 @@
       <c r="B31" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="1" t="s">
         <v>332</v>
       </c>
       <c r="D31" t="s">
@@ -2418,7 +2417,7 @@
       <c r="B32" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="1" t="s">
         <v>357</v>
       </c>
       <c r="D32" t="s">
@@ -2447,7 +2446,7 @@
       <c r="B33" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="1" t="s">
         <v>335</v>
       </c>
       <c r="D33" t="s">
@@ -2476,7 +2475,7 @@
       <c r="B34" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="1" t="s">
         <v>322</v>
       </c>
       <c r="D34" t="s">
@@ -2505,7 +2504,7 @@
       <c r="B35" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C35" s="1" t="s">
         <v>325</v>
       </c>
       <c r="D35" t="s">
@@ -2534,7 +2533,7 @@
       <c r="B36" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="1" t="s">
         <v>345</v>
       </c>
       <c r="D36" t="s">
@@ -2563,7 +2562,7 @@
       <c r="B37" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="1" t="s">
         <v>317</v>
       </c>
       <c r="D37" t="s">
@@ -2592,7 +2591,7 @@
       <c r="B38" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="1" t="s">
         <v>316</v>
       </c>
       <c r="D38" t="s">
@@ -2621,7 +2620,7 @@
       <c r="B39" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="1" t="s">
         <v>329</v>
       </c>
       <c r="D39" t="s">
@@ -2650,7 +2649,7 @@
       <c r="B40" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="C40" s="1" t="s">
         <v>339</v>
       </c>
       <c r="D40" t="s">
@@ -2679,7 +2678,7 @@
       <c r="B41" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="1" t="s">
         <v>340</v>
       </c>
       <c r="D41" t="s">
@@ -2708,7 +2707,7 @@
       <c r="B42" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="C42" s="1" t="s">
         <v>353</v>
       </c>
       <c r="D42" t="s">
@@ -2737,7 +2736,7 @@
       <c r="B43" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="C43" s="1" t="s">
         <v>354</v>
       </c>
       <c r="D43" t="s">
@@ -2766,7 +2765,7 @@
       <c r="B44" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="C44" s="1" t="s">
         <v>355</v>
       </c>
       <c r="D44" t="s">
@@ -2795,7 +2794,7 @@
       <c r="B45" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C45" s="1" t="s">
         <v>311</v>
       </c>
       <c r="D45" t="s">
@@ -2824,7 +2823,7 @@
       <c r="B46" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="C46" s="1" t="s">
         <v>330</v>
       </c>
       <c r="D46" t="s">
@@ -2853,7 +2852,7 @@
       <c r="B47" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="C47" s="1" t="s">
         <v>323</v>
       </c>
       <c r="D47" t="s">
@@ -2882,7 +2881,7 @@
       <c r="B48" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C48" s="5" t="s">
+      <c r="C48" s="1" t="s">
         <v>314</v>
       </c>
       <c r="D48" t="s">

</xml_diff>